<commit_message>
Add Vocab Lesson 18
</commit_message>
<xml_diff>
--- a/data/2026_S_F_Vocab.xlsx
+++ b/data/2026_S_F_Vocab.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC3BB828-12F5-4684-B4B3-3601E097FFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4904A3-6D82-4B25-A905-AD2BE8508D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3752CCC5-FE16-4685-BBA0-17C486BBF170}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3752CCC5-FE16-4685-BBA0-17C486BBF170}"/>
   </bookViews>
   <sheets>
     <sheet name="Lesson 17" sheetId="5" r:id="rId1"/>
+    <sheet name="Lesson 18" sheetId="6" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -180,6 +181,96 @@
   </si>
   <si>
     <t>The crops will wither unless we have rain soon.</t>
+  </si>
+  <si>
+    <t>animated</t>
+  </si>
+  <si>
+    <t>adj. 1. Alive or seeming to be alive. 2. Full of energy; lively.</t>
+  </si>
+  <si>
+    <t>betray</t>
+  </si>
+  <si>
+    <t>v. 1. To be disloyal to. 2. To show; to reveal.</t>
+  </si>
+  <si>
+    <t>convince</t>
+  </si>
+  <si>
+    <t>v. To make someone feel sure or certain; to persuade.</t>
+  </si>
+  <si>
+    <t>decline</t>
+  </si>
+  <si>
+    <t>v. 1. To slope or pass to a lower level. 2. To refuse to accept. 3. To become less or weaker. n. 1. A change to a smaller amount or lower level. 2. A loss of strength or power.</t>
+  </si>
+  <si>
+    <t>hilarious</t>
+  </si>
+  <si>
+    <t>adj. Very funny.</t>
+  </si>
+  <si>
+    <t>likeness</t>
+  </si>
+  <si>
+    <t>n. The state of being similar; something that is similar.</t>
+  </si>
+  <si>
+    <t>meager</t>
+  </si>
+  <si>
+    <t>adj. Poor in quality or insufficient in amount.</t>
+  </si>
+  <si>
+    <t>mischief</t>
+  </si>
+  <si>
+    <t>n. 1. Harm or damage. 2. Behavior that causes harm or trouble. 3. Playfulness; harmless amusement.</t>
+  </si>
+  <si>
+    <t>negotiate</t>
+  </si>
+  <si>
+    <t>v. 1. To arrange by talking over. 2. To travel successfully along or over.</t>
+  </si>
+  <si>
+    <t>obsolete</t>
+  </si>
+  <si>
+    <t>adj. No longer sold or in wide use because it is out-of-date.</t>
+  </si>
+  <si>
+    <t>retain</t>
+  </si>
+  <si>
+    <t>v. 1. To hold on to; to keep possession of. 2. To hire the services of.</t>
+  </si>
+  <si>
+    <t>sensation</t>
+  </si>
+  <si>
+    <t>n. 1. A feeling that comes from stimulation of the senses. 2. A feeling of great interest or excitement or the cause of such a feeling.</t>
+  </si>
+  <si>
+    <t>somber</t>
+  </si>
+  <si>
+    <t>adj. 1. Dark; gloomy. 2. Sad; serious.</t>
+  </si>
+  <si>
+    <t>subsequent</t>
+  </si>
+  <si>
+    <t>adj. Coming later; following.</t>
+  </si>
+  <si>
+    <t>vow</t>
+  </si>
+  <si>
+    <t>v. To promise seriously. n. A pledge; a promise.</t>
   </si>
 </sst>
 </file>
@@ -799,4 +890,147 @@
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF73B841-A7C8-48B9-BC70-6CB02660EAD8}">
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="47" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="54" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add vocab Lesson 19
</commit_message>
<xml_diff>
--- a/data/2026_S_F_Vocab.xlsx
+++ b/data/2026_S_F_Vocab.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4B823A-306F-46FD-8A48-1615DB2675C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{014816C0-DA43-442C-93B2-C968CA3E38DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3752CCC5-FE16-4685-BBA0-17C486BBF170}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3752CCC5-FE16-4685-BBA0-17C486BBF170}"/>
   </bookViews>
   <sheets>
     <sheet name="Lesson 17" sheetId="5" r:id="rId1"/>
     <sheet name="Lesson 18" sheetId="6" r:id="rId2"/>
+    <sheet name="Lesson 19" sheetId="7" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="124">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -286,6 +287,136 @@
   </si>
   <si>
     <t>a. 1. Causing great curiosity and interest. 2. very great or excellent.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>단어</t>
+  </si>
+  <si>
+    <t>교재에 나온 뜻</t>
+  </si>
+  <si>
+    <t>dormant</t>
+  </si>
+  <si>
+    <t>adj. 1. In a sleeplike state. 2. Not active, but able to become active.</t>
+  </si>
+  <si>
+    <t>elegant</t>
+  </si>
+  <si>
+    <t>adj. Graceful or refined in appearance or behavior.</t>
+  </si>
+  <si>
+    <t>erupt</t>
+  </si>
+  <si>
+    <t>excavate</t>
+  </si>
+  <si>
+    <t>expel</t>
+  </si>
+  <si>
+    <t>v. 1. To eject; to release, as from a container. 2. To force to leave.</t>
+  </si>
+  <si>
+    <t>fume</t>
+  </si>
+  <si>
+    <t>n. (usually plural) A disagreeable smoke or gas. v. To feel or show anger or resentment.</t>
+  </si>
+  <si>
+    <t>painstaking</t>
+  </si>
+  <si>
+    <t>adj. Showing or taking great care or effort.</t>
+  </si>
+  <si>
+    <t>perish</t>
+  </si>
+  <si>
+    <t>v. To die; to be killed or destroyed.</t>
+  </si>
+  <si>
+    <t>population</t>
+  </si>
+  <si>
+    <t>scald</t>
+  </si>
+  <si>
+    <t>stupendous</t>
+  </si>
+  <si>
+    <t>adj. Amazing because it is very great or very large.</t>
+  </si>
+  <si>
+    <t>suffocate</t>
+  </si>
+  <si>
+    <t>tremor</t>
+  </si>
+  <si>
+    <t>n. 1. A shaking movement. 2. A nervous or excited feeling.</t>
+  </si>
+  <si>
+    <t>eruption</t>
+  </si>
+  <si>
+    <t>excavation</t>
+  </si>
+  <si>
+    <t>populate</t>
+  </si>
+  <si>
+    <t>scalding</t>
+  </si>
+  <si>
+    <t>suffocation</t>
+  </si>
+  <si>
+    <t>v. To burst forth violently.</t>
+  </si>
+  <si>
+    <t>n. A violent bursting forth.</t>
+  </si>
+  <si>
+    <t>v. 1. To dig out. 2. To uncover by digging.</t>
+  </si>
+  <si>
+    <t>n. The place formed by digging or the process of digging out.</t>
+  </si>
+  <si>
+    <t>n. 1. The total number of people in a certain place. 2. The total number of plants or animals in a certain area.</t>
+  </si>
+  <si>
+    <t>v. To fill; to form the population of.</t>
+  </si>
+  <si>
+    <t>v. To burn with hot liquid or steam.</t>
+  </si>
+  <si>
+    <t>adj. Very hot.</t>
+  </si>
+  <si>
+    <t>v. To kill or die by stopping access to air.</t>
+  </si>
+  <si>
+    <t>n. The act or process of suffocating.</t>
+  </si>
+  <si>
+    <t>molten</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. Made liquid by heat; melted.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>prelude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 1. Something that comes before or introduces the main part. 2. A short musical piece played as an introduction.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -364,7 +495,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -382,6 +513,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1065,4 +1202,187 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BB1817-8468-478A-BD83-74FDB293160C}">
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="47" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="33" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Vocab Chapter 20
</commit_message>
<xml_diff>
--- a/data/2026_S_F_Vocab.xlsx
+++ b/data/2026_S_F_Vocab.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{014816C0-DA43-442C-93B2-C968CA3E38DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DE0B3E9-9BE6-4D72-999F-FFE4EA529E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3752CCC5-FE16-4685-BBA0-17C486BBF170}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3752CCC5-FE16-4685-BBA0-17C486BBF170}"/>
   </bookViews>
   <sheets>
     <sheet name="Lesson 17" sheetId="5" r:id="rId1"/>
     <sheet name="Lesson 18" sheetId="6" r:id="rId2"/>
     <sheet name="Lesson 19" sheetId="7" r:id="rId3"/>
+    <sheet name="Lesson 20" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="162">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -417,6 +418,128 @@
   </si>
   <si>
     <t>n. 1. Something that comes before or introduces the main part. 2. A short musical piece played as an introduction.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ample</t>
+  </si>
+  <si>
+    <t>burden</t>
+  </si>
+  <si>
+    <t>compassion</t>
+  </si>
+  <si>
+    <t>compassionate</t>
+  </si>
+  <si>
+    <t>comply</t>
+  </si>
+  <si>
+    <t>cumbersome</t>
+  </si>
+  <si>
+    <t>distress</t>
+  </si>
+  <si>
+    <t>encounter</t>
+  </si>
+  <si>
+    <t>exertion</t>
+  </si>
+  <si>
+    <t>indignant</t>
+  </si>
+  <si>
+    <t>indignation</t>
+  </si>
+  <si>
+    <t>jest</t>
+  </si>
+  <si>
+    <t>outskirts</t>
+  </si>
+  <si>
+    <t>resume</t>
+  </si>
+  <si>
+    <t>ridicule</t>
+  </si>
+  <si>
+    <t>ridiculous</t>
+  </si>
+  <si>
+    <t>adj. 1. Plenty; more than enough. 2. Large in size.</t>
+  </si>
+  <si>
+    <t>n. 1. Something that is carried, especially a heavy load. 2. Anything that is hard to bear. v. To add to what one has to bear.</t>
+  </si>
+  <si>
+    <t>n. A feeling of sharing the suffering of others and of wanting to help; sympathy; pity.</t>
+  </si>
+  <si>
+    <t>adj. The state of showing compassion.</t>
+  </si>
+  <si>
+    <t>v. To act in agreement with a rule or another's wishes.</t>
+  </si>
+  <si>
+    <t>adj. Awkward and hard to handle; unwieldy.</t>
+  </si>
+  <si>
+    <t>v. To cause pain or sorrow; to trouble or worry. n. Pain, sorrow, or worry.</t>
+  </si>
+  <si>
+    <t>v. 1. To meet unexpectedly. 2. To be faced with. n. 1. A chance meeting. 2. A battle or fight.</t>
+  </si>
+  <si>
+    <t>n. The act of tiring oneself; a strong effort.</t>
+  </si>
+  <si>
+    <t>adj. Angry or resentful about something that seems wrong or unfair.</t>
+  </si>
+  <si>
+    <t>n. Anger that is caused by something mean or unfair.</t>
+  </si>
+  <si>
+    <t>n. A joke or the act of joking. v. To joke or say things lightheartedly.</t>
+  </si>
+  <si>
+    <t>n. The parts far from the center, as of a town.</t>
+  </si>
+  <si>
+    <t>v. 1. To begin again after a pause. 2. To occupy again.</t>
+  </si>
+  <si>
+    <t>v. To make fun of; to mock. n. Words or actions intended to make fun of or mock.</t>
+  </si>
+  <si>
+    <t>adj. Laughable; deserving of mockery.</t>
+  </si>
+  <si>
+    <t>exert</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. To put forth effort.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>mirth</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. Laughter; joyfulness expressed through laughter.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>moral</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">n. A useful lesson about life. 
+adj. 1. Having to do with questions of right and wrong. 
+2. Based on what is right and proper. </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1385,4 +1508,179 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A55D91C-6E69-4242-BB6E-D1742F760D86}">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="47" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>